<commit_message>
Marks sheet: failure cases in Classes 3-10
</commit_message>
<xml_diff>
--- a/results/onxxgawftv.xlsx
+++ b/results/onxxgawftv.xlsx
@@ -2289,20 +2289,20 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>35</v>
+        <v>95</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>94</v>
+        <v>40</v>
       </c>
       <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="3" t="n">
-        <v>44</v>
+        <v>97</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>41</v>
+        <v>85</v>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr"/>
@@ -2321,24 +2321,24 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Dimpi Hazarika</t>
+          <t>Dimpi Mahanta</t>
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>52</v>
+        <v>77</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="G53" s="2" t="inlineStr"/>
       <c r="H53" s="3" t="n">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>42</v>
+        <v>84</v>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
       <c r="K53" s="2" t="inlineStr"/>
@@ -2364,17 +2364,17 @@
         <v>53</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="3" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I54" s="3" t="n">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr"/>
@@ -2393,24 +2393,24 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Ankita Nath</t>
+          <t>Karabi Kakati</t>
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>98</v>
+        <v>57</v>
       </c>
       <c r="G55" s="2" t="inlineStr"/>
       <c r="H55" s="3" t="n">
-        <v>52</v>
+        <v>88</v>
       </c>
       <c r="I55" s="3" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="J55" s="2" t="inlineStr"/>
       <c r="K55" s="2" t="inlineStr"/>
@@ -2429,24 +2429,24 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Priya Talukdar</t>
+          <t>Jyotirmoy Nath</t>
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="3" t="n">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="I56" s="3" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J56" s="2" t="inlineStr"/>
       <c r="K56" s="2" t="inlineStr"/>
@@ -2465,24 +2465,24 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Partha Rabha</t>
+          <t>Sangita Sharma</t>
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G57" s="2" t="inlineStr"/>
       <c r="H57" s="3" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="I57" s="3" t="n">
-        <v>98</v>
+        <v>60</v>
       </c>
       <c r="J57" s="2" t="inlineStr"/>
       <c r="K57" s="2" t="inlineStr"/>
@@ -2501,24 +2501,24 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Trishna Boro</t>
+          <t>Gitika Baruah</t>
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="G58" s="2" t="inlineStr"/>
       <c r="H58" s="3" t="n">
-        <v>41</v>
+        <v>70</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="J58" s="2" t="inlineStr"/>
       <c r="K58" s="2" t="inlineStr"/>
@@ -2537,24 +2537,24 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Pooja Boro</t>
+          <t>Ankita Nath</t>
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>40</v>
+        <v>76</v>
       </c>
       <c r="G59" s="2" t="inlineStr"/>
       <c r="H59" s="3" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="I59" s="3" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J59" s="2" t="inlineStr"/>
       <c r="K59" s="2" t="inlineStr"/>
@@ -2573,24 +2573,24 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Sourav Gogoi</t>
+          <t>Rituparna Mahanta</t>
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="3" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="I60" s="3" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" s="2" t="inlineStr"/>
@@ -2609,24 +2609,24 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Pooja Sarmah</t>
+          <t>Priya Mahanta</t>
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="G61" s="2" t="inlineStr"/>
       <c r="H61" s="3" t="n">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="I61" s="3" t="n">
-        <v>58</v>
+        <v>90</v>
       </c>
       <c r="J61" s="2" t="inlineStr"/>
       <c r="K61" s="2" t="inlineStr"/>
@@ -2645,24 +2645,24 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Ankita Saikia</t>
+          <t>Pooja Hazarika</t>
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>38</v>
+        <v>91</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G62" s="2" t="inlineStr"/>
       <c r="H62" s="3" t="n">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="J62" s="2" t="inlineStr"/>
       <c r="K62" s="2" t="inlineStr"/>
@@ -2681,24 +2681,24 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Bikash Talukdar</t>
+          <t>Ankita Boro</t>
         </is>
       </c>
       <c r="D63" s="3" t="n">
         <v>48</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="G63" s="2" t="inlineStr"/>
       <c r="H63" s="3" t="n">
-        <v>84</v>
+        <v>57</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="J63" s="2" t="inlineStr"/>
       <c r="K63" s="2" t="inlineStr"/>
@@ -2717,24 +2717,24 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Mitali Bhattacharya</t>
+          <t>Partha Rabha</t>
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="G64" s="2" t="inlineStr"/>
       <c r="H64" s="3" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="J64" s="2" t="inlineStr"/>
       <c r="K64" s="2" t="inlineStr"/>
@@ -2753,24 +2753,24 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Dimpi Rabha</t>
+          <t>Barnali Hazarika</t>
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G65" s="2" t="inlineStr"/>
       <c r="H65" s="3" t="n">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="I65" s="3" t="n">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="J65" s="2" t="inlineStr"/>
       <c r="K65" s="2" t="inlineStr"/>
@@ -2789,24 +2789,24 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Bikash Rabha</t>
+          <t>Rimjim Sarmah</t>
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G66" s="2" t="inlineStr"/>
       <c r="H66" s="3" t="n">
-        <v>18</v>
+        <v>95</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="J66" s="2" t="inlineStr"/>
       <c r="K66" s="2" t="inlineStr"/>
@@ -2825,24 +2825,24 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Pallabi Boro</t>
+          <t>Sourav Gogoi</t>
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="G67" s="2" t="inlineStr"/>
       <c r="H67" s="3" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="I67" s="3" t="n">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="J67" s="2" t="inlineStr"/>
       <c r="K67" s="2" t="inlineStr"/>
@@ -2861,24 +2861,24 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Karabi Baruah</t>
+          <t>Anaya Kakati</t>
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>82</v>
+        <v>43</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="G68" s="2" t="inlineStr"/>
       <c r="H68" s="3" t="n">
-        <v>28</v>
+        <v>72</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="J68" s="2" t="inlineStr"/>
       <c r="K68" s="2" t="inlineStr"/>
@@ -2897,24 +2897,24 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Kasturi Sharma</t>
+          <t>Manash Medhi</t>
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="G69" s="2" t="inlineStr"/>
       <c r="H69" s="3" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I69" s="3" t="n">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="J69" s="2" t="inlineStr"/>
       <c r="K69" s="2" t="inlineStr"/>
@@ -2933,24 +2933,24 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Pooja Bhattacharya</t>
+          <t>Pranjal Baruah</t>
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>23</v>
+        <v>85</v>
       </c>
       <c r="F70" s="3" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="G70" s="2" t="inlineStr"/>
       <c r="H70" s="3" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="I70" s="3" t="n">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="J70" s="2" t="inlineStr"/>
       <c r="K70" s="2" t="inlineStr"/>
@@ -2969,24 +2969,24 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Partha Bora</t>
+          <t>Dipankar Sarmah</t>
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="G71" s="2" t="inlineStr"/>
       <c r="H71" s="3" t="n">
-        <v>29</v>
+        <v>82</v>
       </c>
       <c r="I71" s="3" t="n">
-        <v>27</v>
+        <v>94</v>
       </c>
       <c r="J71" s="2" t="inlineStr"/>
       <c r="K71" s="2" t="inlineStr"/>
@@ -3005,24 +3005,24 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Juri Kakati</t>
+          <t>Rupam Gogoi</t>
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>54</v>
+        <v>90</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G72" s="2" t="inlineStr"/>
       <c r="H72" s="3" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="I72" s="3" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="J72" s="2" t="inlineStr"/>
       <c r="K72" s="2" t="inlineStr"/>
@@ -3041,24 +3041,24 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Dhruba Nath</t>
+          <t>Anaya Kalita</t>
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="G73" s="2" t="inlineStr"/>
       <c r="H73" s="3" t="n">
-        <v>46</v>
+        <v>87</v>
       </c>
       <c r="I73" s="3" t="n">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="J73" s="2" t="inlineStr"/>
       <c r="K73" s="2" t="inlineStr"/>
@@ -3077,24 +3077,24 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Rupam Bhattacharya</t>
+          <t>Rituparna Saikia</t>
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="G74" s="2" t="inlineStr"/>
       <c r="H74" s="3" t="n">
-        <v>91</v>
+        <v>54</v>
       </c>
       <c r="I74" s="3" t="n">
-        <v>98</v>
+        <v>62</v>
       </c>
       <c r="J74" s="2" t="inlineStr"/>
       <c r="K74" s="2" t="inlineStr"/>
@@ -3113,24 +3113,24 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Manash Hazarika</t>
+          <t>Mitali Hazarika</t>
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="E75" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="F75" s="3" t="n">
         <v>80</v>
-      </c>
-      <c r="F75" s="3" t="n">
-        <v>96</v>
       </c>
       <c r="G75" s="2" t="inlineStr"/>
       <c r="H75" s="3" t="n">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="I75" s="3" t="n">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="J75" s="2" t="inlineStr"/>
       <c r="K75" s="2" t="inlineStr"/>
@@ -3149,24 +3149,24 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Trishna Medhi</t>
+          <t>Chayan Dutta</t>
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F76" s="3" t="n">
         <v>85</v>
       </c>
       <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="3" t="n">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="I76" s="3" t="n">
-        <v>26</v>
+        <v>85</v>
       </c>
       <c r="J76" s="2" t="inlineStr"/>
       <c r="K76" s="2" t="inlineStr"/>
@@ -3185,24 +3185,24 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Hirak Choudhury</t>
+          <t>Dimpi Saikia</t>
         </is>
       </c>
       <c r="D77" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="E77" s="3" t="n">
+        <v>71</v>
+      </c>
+      <c r="F77" s="3" t="n">
         <v>79</v>
-      </c>
-      <c r="E77" s="3" t="n">
-        <v>76</v>
-      </c>
-      <c r="F77" s="3" t="n">
-        <v>66</v>
       </c>
       <c r="G77" s="2" t="inlineStr"/>
       <c r="H77" s="3" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="I77" s="3" t="n">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="J77" s="2" t="inlineStr"/>
       <c r="K77" s="2" t="inlineStr"/>
@@ -3221,24 +3221,24 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Nirupama Bhattacharya</t>
+          <t>Mamoni Saikia</t>
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>39</v>
+        <v>87</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>98</v>
+        <v>61</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="3" t="n">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="I78" s="3" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="J78" s="2" t="inlineStr"/>
       <c r="K78" s="2" t="inlineStr"/>
@@ -3257,24 +3257,24 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Trishna Sharma</t>
+          <t>Nirupama Medhi</t>
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="G79" s="2" t="inlineStr"/>
       <c r="H79" s="3" t="n">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="I79" s="3" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="J79" s="2" t="inlineStr"/>
       <c r="K79" s="2" t="inlineStr"/>
@@ -3293,24 +3293,24 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Rima Boro</t>
+          <t>Aarav Sarmah</t>
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="E80" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="F80" s="3" t="n">
         <v>52</v>
-      </c>
-      <c r="F80" s="3" t="n">
-        <v>34</v>
       </c>
       <c r="G80" s="2" t="inlineStr"/>
       <c r="H80" s="3" t="n">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="I80" s="3" t="n">
-        <v>37</v>
+        <v>79</v>
       </c>
       <c r="J80" s="2" t="inlineStr"/>
       <c r="K80" s="2" t="inlineStr"/>
@@ -3329,21 +3329,21 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Utpal Sarmah</t>
+          <t>Himangshu Dutta</t>
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>87</v>
+        <v>46</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="G81" s="2" t="inlineStr"/>
       <c r="H81" s="3" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="I81" s="3" t="n">
         <v>66</v>
@@ -3365,28 +3365,28 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Karabi Saikia</t>
+          <t>Anaya Rabha</t>
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="G82" s="2" t="inlineStr"/>
       <c r="H82" s="2" t="inlineStr"/>
       <c r="I82" s="3" t="n">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="J82" s="3" t="n">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="L82" s="2" t="inlineStr"/>
       <c r="M82" s="2" t="inlineStr"/>
@@ -3403,28 +3403,28 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Himangshu Dutta</t>
+          <t>Jyotirmoy Kalita</t>
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>28</v>
+        <v>73</v>
       </c>
       <c r="E83" s="3" t="n">
         <v>85</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="G83" s="2" t="inlineStr"/>
       <c r="H83" s="2" t="inlineStr"/>
       <c r="I83" s="3" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J83" s="3" t="n">
+        <v>76</v>
+      </c>
+      <c r="K83" s="3" t="n">
         <v>89</v>
-      </c>
-      <c r="K83" s="3" t="n">
-        <v>67</v>
       </c>
       <c r="L83" s="2" t="inlineStr"/>
       <c r="M83" s="2" t="inlineStr"/>
@@ -3441,28 +3441,28 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Pranjal Rabha</t>
+          <t>Abhijit Choudhury</t>
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>19</v>
+        <v>93</v>
       </c>
       <c r="G84" s="2" t="inlineStr"/>
       <c r="H84" s="2" t="inlineStr"/>
       <c r="I84" s="3" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="J84" s="3" t="n">
-        <v>59</v>
+        <v>91</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="L84" s="2" t="inlineStr"/>
       <c r="M84" s="2" t="inlineStr"/>
@@ -3479,28 +3479,28 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Rahul Kalita</t>
+          <t>Pallabi Dutta</t>
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G85" s="2" t="inlineStr"/>
       <c r="H85" s="2" t="inlineStr"/>
       <c r="I85" s="3" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="J85" s="3" t="n">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>35</v>
+        <v>98</v>
       </c>
       <c r="L85" s="2" t="inlineStr"/>
       <c r="M85" s="2" t="inlineStr"/>
@@ -3517,28 +3517,28 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Utpal Bora</t>
+          <t>Chayan Sarmah</t>
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>76</v>
+        <v>41</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="G86" s="2" t="inlineStr"/>
       <c r="H86" s="2" t="inlineStr"/>
       <c r="I86" s="3" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="J86" s="3" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="L86" s="2" t="inlineStr"/>
       <c r="M86" s="2" t="inlineStr"/>
@@ -3555,28 +3555,28 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Sourav Sarmah</t>
+          <t>Rima Medhi</t>
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="G87" s="2" t="inlineStr"/>
       <c r="H87" s="2" t="inlineStr"/>
       <c r="I87" s="3" t="n">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="J87" s="3" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="L87" s="2" t="inlineStr"/>
       <c r="M87" s="2" t="inlineStr"/>
@@ -3593,17 +3593,17 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Dimpi Medhi</t>
+          <t>Pallabi Bhattacharya</t>
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E88" s="3" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>18</v>
+        <v>85</v>
       </c>
       <c r="G88" s="2" t="inlineStr"/>
       <c r="H88" s="2" t="inlineStr"/>
@@ -3611,10 +3611,10 @@
         <v>74</v>
       </c>
       <c r="J88" s="3" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="L88" s="2" t="inlineStr"/>
       <c r="M88" s="2" t="inlineStr"/>
@@ -3631,28 +3631,28 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Manash Mahanta</t>
+          <t>Rupam Choudhury</t>
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="G89" s="2" t="inlineStr"/>
       <c r="H89" s="2" t="inlineStr"/>
       <c r="I89" s="3" t="n">
-        <v>21</v>
+        <v>73</v>
       </c>
       <c r="J89" s="3" t="n">
-        <v>53</v>
+        <v>89</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="L89" s="2" t="inlineStr"/>
       <c r="M89" s="2" t="inlineStr"/>
@@ -3669,28 +3669,28 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Utpal Saikia</t>
+          <t>Abhijit Bora</t>
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>52</v>
+        <v>96</v>
       </c>
       <c r="E90" s="3" t="n">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="G90" s="2" t="inlineStr"/>
       <c r="H90" s="2" t="inlineStr"/>
       <c r="I90" s="3" t="n">
-        <v>91</v>
+        <v>42</v>
       </c>
       <c r="J90" s="3" t="n">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>83</v>
+        <v>49</v>
       </c>
       <c r="L90" s="2" t="inlineStr"/>
       <c r="M90" s="2" t="inlineStr"/>
@@ -3707,28 +3707,28 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Mamoni Talukdar</t>
+          <t>Barnali Deka</t>
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="E91" s="3" t="n">
-        <v>21</v>
+        <v>89</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="G91" s="2" t="inlineStr"/>
       <c r="H91" s="2" t="inlineStr"/>
       <c r="I91" s="3" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J91" s="3" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="L91" s="2" t="inlineStr"/>
       <c r="M91" s="2" t="inlineStr"/>
@@ -3745,28 +3745,28 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Mamoni Medhi</t>
+          <t>Sumi Boro</t>
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>24</v>
+        <v>87</v>
       </c>
       <c r="E92" s="3" t="n">
-        <v>54</v>
+        <v>94</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G92" s="2" t="inlineStr"/>
       <c r="H92" s="2" t="inlineStr"/>
       <c r="I92" s="3" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J92" s="3" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="L92" s="2" t="inlineStr"/>
       <c r="M92" s="2" t="inlineStr"/>
@@ -3783,17 +3783,17 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Abhijit Choudhury</t>
+          <t>Rahul Medhi</t>
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="E93" s="3" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
       <c r="H93" s="2" t="inlineStr"/>
@@ -3801,10 +3801,10 @@
         <v>52</v>
       </c>
       <c r="J93" s="3" t="n">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="L93" s="2" t="inlineStr"/>
       <c r="M93" s="2" t="inlineStr"/>
@@ -3821,28 +3821,28 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Rituparna Hazarika</t>
+          <t>Priya Hazarika</t>
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="E94" s="3" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>80</v>
+        <v>48</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
       <c r="H94" s="2" t="inlineStr"/>
       <c r="I94" s="3" t="n">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="J94" s="3" t="n">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="K94" s="3" t="n">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="L94" s="2" t="inlineStr"/>
       <c r="M94" s="2" t="inlineStr"/>
@@ -3859,28 +3859,28 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Hirak Medhi</t>
+          <t>Rima Gogoi</t>
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>27</v>
+        <v>85</v>
       </c>
       <c r="E95" s="3" t="n">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>65</v>
+        <v>97</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
       <c r="H95" s="2" t="inlineStr"/>
       <c r="I95" s="3" t="n">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="J95" s="3" t="n">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="K95" s="3" t="n">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="L95" s="2" t="inlineStr"/>
       <c r="M95" s="2" t="inlineStr"/>
@@ -3897,28 +3897,28 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Utpal Deka</t>
+          <t>Himangshu Hazarika</t>
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="E96" s="3" t="n">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="F96" s="3" t="n">
-        <v>92</v>
+        <v>45</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
       <c r="H96" s="2" t="inlineStr"/>
       <c r="I96" s="3" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="J96" s="3" t="n">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="K96" s="3" t="n">
-        <v>43</v>
+        <v>76</v>
       </c>
       <c r="L96" s="2" t="inlineStr"/>
       <c r="M96" s="2" t="inlineStr"/>
@@ -3935,28 +3935,28 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Sumi Dutta</t>
+          <t>Mintu Bora</t>
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>97</v>
+        <v>50</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>80</v>
+        <v>54</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="G97" s="2" t="inlineStr"/>
       <c r="H97" s="2" t="inlineStr"/>
       <c r="I97" s="3" t="n">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J97" s="3" t="n">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="K97" s="3" t="n">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="L97" s="2" t="inlineStr"/>
       <c r="M97" s="2" t="inlineStr"/>
@@ -3973,28 +3973,28 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Juri Sharma</t>
+          <t>Utpal Mahanta</t>
         </is>
       </c>
       <c r="D98" s="3" t="n">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="G98" s="2" t="inlineStr"/>
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="3" t="n">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="J98" s="3" t="n">
-        <v>47</v>
+        <v>87</v>
       </c>
       <c r="K98" s="3" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="L98" s="2" t="inlineStr"/>
       <c r="M98" s="2" t="inlineStr"/>
@@ -4011,28 +4011,28 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Kangkan Dutta</t>
+          <t>Pranjal Das</t>
         </is>
       </c>
       <c r="D99" s="3" t="n">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>44</v>
+        <v>89</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="G99" s="2" t="inlineStr"/>
       <c r="H99" s="2" t="inlineStr"/>
       <c r="I99" s="3" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="J99" s="3" t="n">
-        <v>36</v>
+        <v>95</v>
       </c>
       <c r="K99" s="3" t="n">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="L99" s="2" t="inlineStr"/>
       <c r="M99" s="2" t="inlineStr"/>
@@ -4049,28 +4049,28 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Sumi Choudhury</t>
+          <t>Dipankar Boro</t>
         </is>
       </c>
       <c r="D100" s="3" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E100" s="3" t="n">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="F100" s="3" t="n">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="G100" s="2" t="inlineStr"/>
       <c r="H100" s="2" t="inlineStr"/>
       <c r="I100" s="3" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J100" s="3" t="n">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="K100" s="3" t="n">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="L100" s="2" t="inlineStr"/>
       <c r="M100" s="2" t="inlineStr"/>
@@ -4087,28 +4087,28 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Kangkan Choudhury</t>
+          <t>Rima Bora</t>
         </is>
       </c>
       <c r="D101" s="3" t="n">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="E101" s="3" t="n">
-        <v>28</v>
+        <v>68</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="G101" s="2" t="inlineStr"/>
       <c r="H101" s="2" t="inlineStr"/>
       <c r="I101" s="3" t="n">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="J101" s="3" t="n">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="K101" s="3" t="n">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="L101" s="2" t="inlineStr"/>
       <c r="M101" s="2" t="inlineStr"/>
@@ -4125,28 +4125,28 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Sourav Boro</t>
+          <t>Manash Hazarika</t>
         </is>
       </c>
       <c r="D102" s="3" t="n">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="E102" s="3" t="n">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G102" s="2" t="inlineStr"/>
       <c r="H102" s="2" t="inlineStr"/>
       <c r="I102" s="3" t="n">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="J102" s="3" t="n">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="K102" s="3" t="n">
-        <v>85</v>
+        <v>22</v>
       </c>
       <c r="L102" s="2" t="inlineStr"/>
       <c r="M102" s="2" t="inlineStr"/>
@@ -4163,28 +4163,28 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Utpal Hazarika</t>
+          <t>Trishna Medhi</t>
         </is>
       </c>
       <c r="D103" s="3" t="n">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="E103" s="3" t="n">
-        <v>37</v>
+        <v>70</v>
       </c>
       <c r="F103" s="3" t="n">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G103" s="2" t="inlineStr"/>
       <c r="H103" s="2" t="inlineStr"/>
       <c r="I103" s="3" t="n">
+        <v>89</v>
+      </c>
+      <c r="J103" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="J103" s="3" t="n">
-        <v>35</v>
-      </c>
       <c r="K103" s="3" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="L103" s="2" t="inlineStr"/>
       <c r="M103" s="2" t="inlineStr"/>
@@ -4201,28 +4201,28 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Rima Das</t>
+          <t>Rupam Medhi</t>
         </is>
       </c>
       <c r="D104" s="3" t="n">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="E104" s="3" t="n">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="F104" s="3" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="G104" s="2" t="inlineStr"/>
       <c r="H104" s="2" t="inlineStr"/>
       <c r="I104" s="3" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="J104" s="3" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="K104" s="3" t="n">
-        <v>87</v>
+        <v>44</v>
       </c>
       <c r="L104" s="2" t="inlineStr"/>
       <c r="M104" s="2" t="inlineStr"/>
@@ -4239,28 +4239,28 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Jyotirmoy Choudhury</t>
+          <t>Rituparna Dutta</t>
         </is>
       </c>
       <c r="D105" s="3" t="n">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="E105" s="3" t="n">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="F105" s="3" t="n">
-        <v>93</v>
+        <v>56</v>
       </c>
       <c r="G105" s="2" t="inlineStr"/>
       <c r="H105" s="2" t="inlineStr"/>
       <c r="I105" s="3" t="n">
-        <v>46</v>
+        <v>95</v>
       </c>
       <c r="J105" s="3" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K105" s="3" t="n">
-        <v>78</v>
+        <v>56</v>
       </c>
       <c r="L105" s="2" t="inlineStr"/>
       <c r="M105" s="2" t="inlineStr"/>
@@ -4277,28 +4277,28 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Rima Sarmah</t>
+          <t>Utpal Bora</t>
         </is>
       </c>
       <c r="D106" s="3" t="n">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="E106" s="3" t="n">
-        <v>36</v>
+        <v>96</v>
       </c>
       <c r="F106" s="3" t="n">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="G106" s="2" t="inlineStr"/>
       <c r="H106" s="2" t="inlineStr"/>
       <c r="I106" s="3" t="n">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="J106" s="3" t="n">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="K106" s="3" t="n">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="L106" s="2" t="inlineStr"/>
       <c r="M106" s="2" t="inlineStr"/>
@@ -4315,28 +4315,28 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Sourav Medhi</t>
+          <t>Nirupama Bhattacharya</t>
         </is>
       </c>
       <c r="D107" s="3" t="n">
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="E107" s="3" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="F107" s="3" t="n">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="G107" s="2" t="inlineStr"/>
       <c r="H107" s="2" t="inlineStr"/>
       <c r="I107" s="3" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="J107" s="3" t="n">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="K107" s="3" t="n">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="L107" s="2" t="inlineStr"/>
       <c r="M107" s="2" t="inlineStr"/>
@@ -4353,28 +4353,28 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Gitika Boro</t>
+          <t>Abhijit Deka</t>
         </is>
       </c>
       <c r="D108" s="3" t="n">
-        <v>61</v>
+        <v>98</v>
       </c>
       <c r="E108" s="3" t="n">
-        <v>50</v>
+        <v>86</v>
       </c>
       <c r="F108" s="3" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G108" s="2" t="inlineStr"/>
       <c r="H108" s="2" t="inlineStr"/>
       <c r="I108" s="3" t="n">
-        <v>48</v>
+        <v>91</v>
       </c>
       <c r="J108" s="3" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K108" s="3" t="n">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="L108" s="2" t="inlineStr"/>
       <c r="M108" s="2" t="inlineStr"/>
@@ -4391,28 +4391,28 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Pooja Baruah</t>
+          <t>Rima Saikia</t>
         </is>
       </c>
       <c r="D109" s="3" t="n">
-        <v>69</v>
+        <v>40</v>
       </c>
       <c r="E109" s="3" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F109" s="3" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G109" s="2" t="inlineStr"/>
       <c r="H109" s="2" t="inlineStr"/>
       <c r="I109" s="3" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="J109" s="3" t="n">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="K109" s="3" t="n">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="L109" s="2" t="inlineStr"/>
       <c r="M109" s="2" t="inlineStr"/>
@@ -4429,28 +4429,28 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Nayan Bora</t>
+          <t>Sangita Das</t>
         </is>
       </c>
       <c r="D110" s="3" t="n">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="E110" s="3" t="n">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="F110" s="3" t="n">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="G110" s="2" t="inlineStr"/>
       <c r="H110" s="2" t="inlineStr"/>
       <c r="I110" s="3" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="J110" s="3" t="n">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="K110" s="3" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="L110" s="2" t="inlineStr"/>
       <c r="M110" s="2" t="inlineStr"/>
@@ -4467,28 +4467,28 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Hirak Saikia</t>
+          <t>Abhijit Sharma</t>
         </is>
       </c>
       <c r="D111" s="3" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>44</v>
+        <v>96</v>
       </c>
       <c r="F111" s="3" t="n">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="G111" s="2" t="inlineStr"/>
       <c r="H111" s="2" t="inlineStr"/>
       <c r="I111" s="3" t="n">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="J111" s="3" t="n">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="K111" s="3" t="n">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="L111" s="2" t="inlineStr"/>
       <c r="M111" s="2" t="inlineStr"/>
@@ -4505,31 +4505,31 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Pranjal Deka</t>
+          <t>Rimjim Deka</t>
         </is>
       </c>
       <c r="D112" s="3" t="n">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="E112" s="3" t="n">
-        <v>77</v>
+        <v>41</v>
       </c>
       <c r="F112" s="3" t="n">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
       <c r="H112" s="2" t="inlineStr"/>
       <c r="I112" s="2" t="inlineStr"/>
       <c r="J112" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="K112" s="3" t="n">
         <v>40</v>
-      </c>
-      <c r="K112" s="3" t="n">
-        <v>25</v>
       </c>
       <c r="L112" s="2" t="inlineStr"/>
       <c r="M112" s="2" t="inlineStr"/>
       <c r="N112" s="3" t="n">
-        <v>66</v>
+        <v>98</v>
       </c>
     </row>
     <row r="113">
@@ -4543,30 +4543,30 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>Karabi Sharma</t>
+          <t>Utpal Sarmah</t>
         </is>
       </c>
       <c r="D113" s="3" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="E113" s="3" t="n">
-        <v>46</v>
+        <v>74</v>
       </c>
       <c r="F113" s="3" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="G113" s="2" t="inlineStr"/>
       <c r="H113" s="2" t="inlineStr"/>
       <c r="I113" s="2" t="inlineStr"/>
       <c r="J113" s="3" t="n">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="K113" s="3" t="n">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="L113" s="2" t="inlineStr"/>
       <c r="M113" s="3" t="n">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="N113" s="2" t="inlineStr"/>
     </row>
@@ -4581,29 +4581,29 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>Jyotirmoy Dutta</t>
+          <t>Manash Talukdar</t>
         </is>
       </c>
       <c r="D114" s="3" t="n">
-        <v>88</v>
+        <v>51</v>
       </c>
       <c r="E114" s="3" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="F114" s="3" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="G114" s="2" t="inlineStr"/>
       <c r="H114" s="2" t="inlineStr"/>
       <c r="I114" s="2" t="inlineStr"/>
       <c r="J114" s="3" t="n">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="K114" s="3" t="n">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="L114" s="3" t="n">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="M114" s="2" t="inlineStr"/>
       <c r="N114" s="2" t="inlineStr"/>
@@ -4619,30 +4619,30 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>Nayan Rabha</t>
+          <t>Trishna Kakati</t>
         </is>
       </c>
       <c r="D115" s="3" t="n">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="E115" s="3" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F115" s="3" t="n">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="G115" s="2" t="inlineStr"/>
       <c r="H115" s="2" t="inlineStr"/>
       <c r="I115" s="2" t="inlineStr"/>
       <c r="J115" s="3" t="n">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="K115" s="3" t="n">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="L115" s="2" t="inlineStr"/>
       <c r="M115" s="3" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="N115" s="2" t="inlineStr"/>
     </row>
@@ -4657,31 +4657,31 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>Sumi Kakati</t>
+          <t>Mamoni Hazarika</t>
         </is>
       </c>
       <c r="D116" s="3" t="n">
-        <v>82</v>
+        <v>27</v>
       </c>
       <c r="E116" s="3" t="n">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="F116" s="3" t="n">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="G116" s="2" t="inlineStr"/>
       <c r="H116" s="2" t="inlineStr"/>
       <c r="I116" s="2" t="inlineStr"/>
       <c r="J116" s="3" t="n">
-        <v>54</v>
+        <v>90</v>
       </c>
       <c r="K116" s="3" t="n">
-        <v>79</v>
-      </c>
-      <c r="L116" s="2" t="inlineStr"/>
-      <c r="M116" s="3" t="n">
-        <v>93</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="L116" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="M116" s="2" t="inlineStr"/>
       <c r="N116" s="2" t="inlineStr"/>
     </row>
     <row r="117">
@@ -4695,31 +4695,31 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>Jyotirmoy Sarmah</t>
+          <t>Mamoni Talukdar</t>
         </is>
       </c>
       <c r="D117" s="3" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E117" s="3" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F117" s="3" t="n">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="G117" s="2" t="inlineStr"/>
       <c r="H117" s="2" t="inlineStr"/>
       <c r="I117" s="2" t="inlineStr"/>
       <c r="J117" s="3" t="n">
-        <v>95</v>
+        <v>56</v>
       </c>
       <c r="K117" s="3" t="n">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="L117" s="2" t="inlineStr"/>
       <c r="M117" s="2" t="inlineStr"/>
       <c r="N117" s="3" t="n">
-        <v>89</v>
+        <v>77</v>
       </c>
     </row>
     <row r="118">
@@ -4733,30 +4733,30 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>Mitali Baruah</t>
+          <t>Partha Saikia</t>
         </is>
       </c>
       <c r="D118" s="3" t="n">
-        <v>18</v>
+        <v>97</v>
       </c>
       <c r="E118" s="3" t="n">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="F118" s="3" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G118" s="2" t="inlineStr"/>
       <c r="H118" s="2" t="inlineStr"/>
       <c r="I118" s="2" t="inlineStr"/>
       <c r="J118" s="3" t="n">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="K118" s="3" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L118" s="2" t="inlineStr"/>
       <c r="M118" s="3" t="n">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="N118" s="2" t="inlineStr"/>
     </row>
@@ -4771,31 +4771,31 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>Nayan Choudhury</t>
+          <t>Pranjal Rabha</t>
         </is>
       </c>
       <c r="D119" s="3" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="E119" s="3" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F119" s="3" t="n">
-        <v>53</v>
+        <v>94</v>
       </c>
       <c r="G119" s="2" t="inlineStr"/>
       <c r="H119" s="2" t="inlineStr"/>
       <c r="I119" s="2" t="inlineStr"/>
       <c r="J119" s="3" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="K119" s="3" t="n">
-        <v>75</v>
-      </c>
-      <c r="L119" s="3" t="n">
-        <v>75</v>
-      </c>
-      <c r="M119" s="2" t="inlineStr"/>
+        <v>43</v>
+      </c>
+      <c r="L119" s="2" t="inlineStr"/>
+      <c r="M119" s="3" t="n">
+        <v>52</v>
+      </c>
       <c r="N119" s="2" t="inlineStr"/>
     </row>
     <row r="120">
@@ -4809,31 +4809,31 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>Dipankar Das</t>
+          <t>Juri Rabha</t>
         </is>
       </c>
       <c r="D120" s="3" t="n">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="E120" s="3" t="n">
-        <v>35</v>
+        <v>89</v>
       </c>
       <c r="F120" s="3" t="n">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="G120" s="2" t="inlineStr"/>
       <c r="H120" s="2" t="inlineStr"/>
       <c r="I120" s="2" t="inlineStr"/>
       <c r="J120" s="3" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="K120" s="3" t="n">
-        <v>81</v>
-      </c>
-      <c r="L120" s="2" t="inlineStr"/>
-      <c r="M120" s="3" t="n">
-        <v>43</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="L120" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="M120" s="2" t="inlineStr"/>
       <c r="N120" s="2" t="inlineStr"/>
     </row>
     <row r="121">
@@ -4847,30 +4847,30 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>Rupam Kakati</t>
+          <t>Rahul Kalita</t>
         </is>
       </c>
       <c r="D121" s="3" t="n">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="E121" s="3" t="n">
-        <v>57</v>
+        <v>89</v>
       </c>
       <c r="F121" s="3" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G121" s="2" t="inlineStr"/>
       <c r="H121" s="2" t="inlineStr"/>
       <c r="I121" s="2" t="inlineStr"/>
       <c r="J121" s="3" t="n">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="K121" s="3" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="L121" s="2" t="inlineStr"/>
       <c r="M121" s="3" t="n">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="N121" s="2" t="inlineStr"/>
     </row>
@@ -4885,31 +4885,31 @@
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>Dimpi Das</t>
+          <t>Gitika Kakati</t>
         </is>
       </c>
       <c r="D122" s="3" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E122" s="3" t="n">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="F122" s="3" t="n">
-        <v>51</v>
+        <v>81</v>
       </c>
       <c r="G122" s="2" t="inlineStr"/>
       <c r="H122" s="2" t="inlineStr"/>
       <c r="I122" s="2" t="inlineStr"/>
       <c r="J122" s="3" t="n">
-        <v>81</v>
+        <v>50</v>
       </c>
       <c r="K122" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="L122" s="2" t="inlineStr"/>
-      <c r="M122" s="3" t="n">
-        <v>78</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="L122" s="3" t="n">
+        <v>71</v>
+      </c>
+      <c r="M122" s="2" t="inlineStr"/>
       <c r="N122" s="2" t="inlineStr"/>
     </row>
     <row r="123">
@@ -4923,31 +4923,31 @@
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>Himangshu Talukdar</t>
+          <t>Nayan Boro</t>
         </is>
       </c>
       <c r="D123" s="3" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E123" s="3" t="n">
-        <v>34</v>
+        <v>93</v>
       </c>
       <c r="F123" s="3" t="n">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="G123" s="2" t="inlineStr"/>
       <c r="H123" s="2" t="inlineStr"/>
       <c r="I123" s="2" t="inlineStr"/>
       <c r="J123" s="3" t="n">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="K123" s="3" t="n">
-        <v>74</v>
-      </c>
-      <c r="L123" s="3" t="n">
-        <v>65</v>
-      </c>
-      <c r="M123" s="2" t="inlineStr"/>
+        <v>72</v>
+      </c>
+      <c r="L123" s="2" t="inlineStr"/>
+      <c r="M123" s="3" t="n">
+        <v>44</v>
+      </c>
       <c r="N123" s="2" t="inlineStr"/>
     </row>
     <row r="124">
@@ -4961,32 +4961,32 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>Jyotirmoy Nath</t>
+          <t>Utpal Hazarika</t>
         </is>
       </c>
       <c r="D124" s="3" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="E124" s="3" t="n">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="F124" s="3" t="n">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="G124" s="2" t="inlineStr"/>
       <c r="H124" s="2" t="inlineStr"/>
       <c r="I124" s="2" t="inlineStr"/>
       <c r="J124" s="3" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="K124" s="3" t="n">
-        <v>86</v>
-      </c>
-      <c r="L124" s="2" t="inlineStr"/>
+        <v>52</v>
+      </c>
+      <c r="L124" s="3" t="n">
+        <v>57</v>
+      </c>
       <c r="M124" s="2" t="inlineStr"/>
-      <c r="N124" s="3" t="n">
-        <v>87</v>
-      </c>
+      <c r="N124" s="2" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -4999,30 +4999,30 @@
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>Barnali Rabha</t>
+          <t>Sourav Sarmah</t>
         </is>
       </c>
       <c r="D125" s="3" t="n">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="E125" s="3" t="n">
-        <v>24</v>
+        <v>92</v>
       </c>
       <c r="F125" s="3" t="n">
-        <v>44</v>
+        <v>86</v>
       </c>
       <c r="G125" s="2" t="inlineStr"/>
       <c r="H125" s="2" t="inlineStr"/>
       <c r="I125" s="2" t="inlineStr"/>
       <c r="J125" s="3" t="n">
-        <v>58</v>
+        <v>80</v>
       </c>
       <c r="K125" s="3" t="n">
-        <v>98</v>
+        <v>71</v>
       </c>
       <c r="L125" s="2" t="inlineStr"/>
       <c r="M125" s="3" t="n">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="N125" s="2" t="inlineStr"/>
     </row>
@@ -5037,31 +5037,31 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>Mitali Deka</t>
+          <t>Mintu Bhattacharya</t>
         </is>
       </c>
       <c r="D126" s="3" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E126" s="3" t="n">
-        <v>74</v>
+        <v>43</v>
       </c>
       <c r="F126" s="3" t="n">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="G126" s="2" t="inlineStr"/>
       <c r="H126" s="2" t="inlineStr"/>
       <c r="I126" s="2" t="inlineStr"/>
       <c r="J126" s="3" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K126" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="L126" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="M126" s="2" t="inlineStr"/>
+        <v>71</v>
+      </c>
+      <c r="L126" s="2" t="inlineStr"/>
+      <c r="M126" s="3" t="n">
+        <v>57</v>
+      </c>
       <c r="N126" s="2" t="inlineStr"/>
     </row>
     <row r="127">
@@ -5075,31 +5075,31 @@
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>Mitali Medhi</t>
+          <t>Dimpi Medhi</t>
         </is>
       </c>
       <c r="D127" s="3" t="n">
-        <v>96</v>
+        <v>53</v>
       </c>
       <c r="E127" s="3" t="n">
-        <v>37</v>
+        <v>87</v>
       </c>
       <c r="F127" s="3" t="n">
-        <v>94</v>
+        <v>66</v>
       </c>
       <c r="G127" s="2" t="inlineStr"/>
       <c r="H127" s="2" t="inlineStr"/>
       <c r="I127" s="2" t="inlineStr"/>
       <c r="J127" s="3" t="n">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="K127" s="3" t="n">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="L127" s="2" t="inlineStr"/>
       <c r="M127" s="2" t="inlineStr"/>
       <c r="N127" s="3" t="n">
-        <v>80</v>
+        <v>51</v>
       </c>
     </row>
     <row r="128">
@@ -5113,14 +5113,14 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>Juri Deka</t>
+          <t>Kaushik Das</t>
         </is>
       </c>
       <c r="D128" s="3" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="E128" s="3" t="n">
-        <v>29</v>
+        <v>69</v>
       </c>
       <c r="F128" s="3" t="n">
         <v>54</v>
@@ -5129,16 +5129,16 @@
       <c r="H128" s="2" t="inlineStr"/>
       <c r="I128" s="2" t="inlineStr"/>
       <c r="J128" s="3" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="K128" s="3" t="n">
-        <v>49</v>
-      </c>
-      <c r="L128" s="2" t="inlineStr"/>
+        <v>88</v>
+      </c>
+      <c r="L128" s="3" t="n">
+        <v>78</v>
+      </c>
       <c r="M128" s="2" t="inlineStr"/>
-      <c r="N128" s="3" t="n">
-        <v>51</v>
-      </c>
+      <c r="N128" s="2" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -5151,30 +5151,30 @@
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>Utpal Das</t>
+          <t>Sangita Talukdar</t>
         </is>
       </c>
       <c r="D129" s="3" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E129" s="3" t="n">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="F129" s="3" t="n">
-        <v>97</v>
+        <v>60</v>
       </c>
       <c r="G129" s="2" t="inlineStr"/>
       <c r="H129" s="2" t="inlineStr"/>
       <c r="I129" s="2" t="inlineStr"/>
       <c r="J129" s="3" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="K129" s="3" t="n">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="L129" s="2" t="inlineStr"/>
       <c r="M129" s="3" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="N129" s="2" t="inlineStr"/>
     </row>
@@ -5189,31 +5189,31 @@
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>Mitali Sharma</t>
+          <t>Hirak Gogoi</t>
         </is>
       </c>
       <c r="D130" s="3" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E130" s="3" t="n">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="F130" s="3" t="n">
-        <v>81</v>
+        <v>38</v>
       </c>
       <c r="G130" s="2" t="inlineStr"/>
       <c r="H130" s="2" t="inlineStr"/>
       <c r="I130" s="2" t="inlineStr"/>
       <c r="J130" s="3" t="n">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="K130" s="3" t="n">
-        <v>91</v>
+        <v>35</v>
       </c>
       <c r="L130" s="2" t="inlineStr"/>
       <c r="M130" s="2" t="inlineStr"/>
       <c r="N130" s="3" t="n">
-        <v>83</v>
+        <v>29</v>
       </c>
     </row>
     <row r="131">
@@ -5227,29 +5227,29 @@
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>Juri Saikia</t>
+          <t>Mintu Deka</t>
         </is>
       </c>
       <c r="D131" s="3" t="n">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="E131" s="3" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F131" s="3" t="n">
-        <v>93</v>
+        <v>56</v>
       </c>
       <c r="G131" s="2" t="inlineStr"/>
       <c r="H131" s="2" t="inlineStr"/>
       <c r="I131" s="2" t="inlineStr"/>
       <c r="J131" s="3" t="n">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="K131" s="3" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="L131" s="3" t="n">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="M131" s="2" t="inlineStr"/>
       <c r="N131" s="2" t="inlineStr"/>

</xml_diff>